<commit_message>
feat: import scripts; color changes
</commit_message>
<xml_diff>
--- a/settlements.xlsx
+++ b/settlements.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="8_{6B50EE4E-0A90-4768-83FE-067AEA81786A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA6D5938-204D-4E35-A13D-F42F6F912714}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{96D043F7-30FF-4798-8320-D73804D07410}"/>
+    <workbookView xWindow="17625" yWindow="2235" windowWidth="11145" windowHeight="11235" xr2:uid="{96D043F7-30FF-4798-8320-D73804D07410}"/>
   </bookViews>
   <sheets>
     <sheet name="settlements" sheetId="1" r:id="rId1"/>
@@ -613,6 +613,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>